<commit_message>
TERMINO EL MODELO POLINOMIAL (Actividad 1 y 2)
</commit_message>
<xml_diff>
--- a/data/Diccionario de datos.xlsx
+++ b/data/Diccionario de datos.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniandes-my.sharepoint.com/personal/mavillam_uniandes_edu_co/Documents/Documentos/cursos/MachineLearning/202620/Laboratorios/lab1/lab1 - copia/datos_laboratorio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6fcf27872eb4cf50/Documentos/UNIANDES/7MO SEMESTRE/APRENDIZAJE DE MAQUINA/LABS/LABORATORIO-2-AM/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_0B4E91BF929C4A4D6962CC35A098F8D7E984A73B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6DF9FB5-839B-435B-B6A8-66D5F2884DB3}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_0B4E91BF929C4A4D6962CC35A098F8D7E984A73B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8697C7E-761D-4850-8B1D-2D0C0305B3EF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -212,12 +225,36 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -232,8 +269,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,14 +578,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
-    <col min="3" max="3" width="103.42578125" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" customWidth="1"/>
+    <col min="3" max="3" width="103.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -555,8 +596,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
@@ -566,8 +607,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
@@ -577,8 +618,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B4" t="s">
@@ -588,8 +629,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B5" t="s">
@@ -599,8 +640,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B6" t="s">
@@ -610,8 +651,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B7" t="s">
@@ -621,8 +662,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B8" t="s">
@@ -632,8 +673,8 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B9" t="s">
@@ -643,8 +684,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B10" t="s">
@@ -654,8 +695,8 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B11" t="s">
@@ -665,8 +706,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B12" t="s">
@@ -676,8 +717,8 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B13" t="s">
@@ -687,8 +728,8 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B14" t="s">
@@ -698,8 +739,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B15" t="s">
@@ -709,8 +750,8 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B16" t="s">
@@ -720,8 +761,8 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B17" t="s">
@@ -731,8 +772,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B18" t="s">
@@ -742,8 +783,8 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B19" t="s">
@@ -753,8 +794,8 @@
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B20" t="s">
@@ -764,8 +805,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B21" t="s">
@@ -775,8 +816,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B22" t="s">
@@ -786,8 +827,8 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B23" t="s">
@@ -797,8 +838,8 @@
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
         <v>49</v>
       </c>
       <c r="B24" t="s">
@@ -808,8 +849,8 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
         <v>51</v>
       </c>
       <c r="B25" t="s">
@@ -819,8 +860,8 @@
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B26" t="s">
@@ -830,8 +871,8 @@
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
         <v>55</v>
       </c>
       <c r="B27" t="s">
@@ -841,8 +882,8 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
         <v>57</v>
       </c>
       <c r="B28" t="s">
@@ -854,5 +895,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>